<commit_message>
Added some changes in dashboad file and pdc transaction report
</commit_message>
<xml_diff>
--- a/PDC Transaction Report.xlsx
+++ b/PDC Transaction Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MCT\Margi - Real Estate Dev\BRE-Property-Management-Margi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{051526AA-6AE5-455A-A1CA-71F4B5041FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{051FFDD7-5810-4DAB-BA3F-0A3EF121836A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
     <definedName name="ReportRequest.TenantId" comment="Use this function to get the Tenant Id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Tenant Id",#REF!,#REF!,"none",)</definedName>
     <definedName name="ReportRequest.UserName" comment="Use this function to get the User name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("User name",#REF!,#REF!,"none",)</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -58,7 +58,7 @@
     <t>Tenant_Id</t>
   </si>
   <si>
-    <t>Tenant_Name_Display</t>
+    <t>Tenant_Name</t>
   </si>
   <si>
     <t>Bank_Name</t>
@@ -171,7 +171,7 @@
     <tableColumn id="3" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="payment_Series"/>
     <tableColumn id="4" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_ID"/>
     <tableColumn id="5" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Tenant_Id"/>
-    <tableColumn id="6" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Tenant_Name_Display"/>
+    <tableColumn id="6" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Tenant_Name"/>
     <tableColumn id="7" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Bank_Name"/>
     <tableColumn id="8" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Cheque_Number"/>
     <tableColumn id="9" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Cheque_Date"/>
@@ -483,18 +483,18 @@
   <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.33203125" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" customWidth="1"/>
-    <col min="3" max="3" width="18.109375" customWidth="1"/>
-    <col min="4" max="4" width="14.6640625" customWidth="1"/>
-    <col min="5" max="5" width="12.77734375" customWidth="1"/>
-    <col min="6" max="6" width="22.33203125" customWidth="1"/>
-    <col min="7" max="7" width="13.77734375" customWidth="1"/>
-    <col min="8" max="8" width="18.5546875" customWidth="1"/>
-    <col min="9" max="9" width="16.6640625" customWidth="1"/>
-    <col min="10" max="10" width="13.6640625" customWidth="1"/>
-    <col min="11" max="11" width="18.21875" customWidth="1"/>
-    <col min="12" max="12" width="17.77734375" customWidth="1"/>
+    <col min="1" max="1" width="31.6640625" customWidth="1"/>
+    <col min="2" max="2" width="12.88671875" customWidth="1"/>
+    <col min="3" max="3" width="18.44140625" customWidth="1"/>
+    <col min="4" max="4" width="14.88671875" customWidth="1"/>
+    <col min="5" max="5" width="14.109375" customWidth="1"/>
+    <col min="6" max="6" width="16.77734375" customWidth="1"/>
+    <col min="7" max="7" width="21.6640625" customWidth="1"/>
+    <col min="8" max="8" width="19.44140625" customWidth="1"/>
+    <col min="9" max="9" width="15.44140625" customWidth="1"/>
+    <col min="10" max="10" width="14.21875" customWidth="1"/>
+    <col min="11" max="11" width="16.33203125" customWidth="1"/>
+    <col min="12" max="12" width="19.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Added a changes in PDC Report
</commit_message>
<xml_diff>
--- a/PDC Transaction Report.xlsx
+++ b/PDC Transaction Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MCT\Margi - Real Estate Dev\BRE-Property-Management-Margi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{051FFDD7-5810-4DAB-BA3F-0A3EF121836A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5480EB3A-E368-478E-AA6A-9DBBAD61E82E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,9 +46,6 @@
     <t>Report_Period</t>
   </si>
   <si>
-    <t>PDC_ID</t>
-  </si>
-  <si>
     <t>payment_Series</t>
   </si>
   <si>
@@ -61,9 +58,6 @@
     <t>Tenant_Name</t>
   </si>
   <si>
-    <t>Bank_Name</t>
-  </si>
-  <si>
     <t>Cheque_Number</t>
   </si>
   <si>
@@ -73,10 +67,16 @@
     <t>Amount</t>
   </si>
   <si>
+    <t>Old_Cheque_</t>
+  </si>
+  <si>
     <t>Cheque_Status</t>
   </si>
   <si>
     <t>Approval_Status</t>
+  </si>
+  <si>
+    <t>Payment_Status</t>
   </si>
   <si>
     <t/>
@@ -167,17 +167,17 @@
   <autoFilter ref="A1:L2" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Report_Period"/>
-    <tableColumn id="2" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="PDC_ID"/>
-    <tableColumn id="3" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="payment_Series"/>
-    <tableColumn id="4" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_ID"/>
-    <tableColumn id="5" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Tenant_Id"/>
-    <tableColumn id="6" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Tenant_Name"/>
-    <tableColumn id="7" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Bank_Name"/>
-    <tableColumn id="8" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Cheque_Number"/>
-    <tableColumn id="9" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Cheque_Date"/>
-    <tableColumn id="10" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Amount"/>
-    <tableColumn id="11" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Cheque_Status"/>
-    <tableColumn id="12" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Approval_Status"/>
+    <tableColumn id="2" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="payment_Series"/>
+    <tableColumn id="3" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_ID"/>
+    <tableColumn id="4" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Tenant_Id"/>
+    <tableColumn id="5" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Tenant_Name"/>
+    <tableColumn id="6" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Cheque_Number"/>
+    <tableColumn id="7" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Cheque_Date"/>
+    <tableColumn id="8" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Amount"/>
+    <tableColumn id="9" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Old_Cheque_"/>
+    <tableColumn id="10" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Cheque_Status"/>
+    <tableColumn id="11" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Approval_Status"/>
+    <tableColumn id="12" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Payment_Status"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -483,18 +483,18 @@
   <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="31.6640625" customWidth="1"/>
-    <col min="2" max="2" width="12.88671875" customWidth="1"/>
-    <col min="3" max="3" width="18.44140625" customWidth="1"/>
-    <col min="4" max="4" width="14.88671875" customWidth="1"/>
-    <col min="5" max="5" width="14.109375" customWidth="1"/>
-    <col min="6" max="6" width="16.77734375" customWidth="1"/>
-    <col min="7" max="7" width="21.6640625" customWidth="1"/>
-    <col min="8" max="8" width="19.44140625" customWidth="1"/>
-    <col min="9" max="9" width="15.44140625" customWidth="1"/>
-    <col min="10" max="10" width="14.21875" customWidth="1"/>
-    <col min="11" max="11" width="16.33203125" customWidth="1"/>
-    <col min="12" max="12" width="19.44140625" customWidth="1"/>
+    <col min="1" max="1" width="26.109375" customWidth="1"/>
+    <col min="2" max="2" width="16.77734375" customWidth="1"/>
+    <col min="3" max="3" width="14.21875" customWidth="1"/>
+    <col min="4" max="4" width="12.109375" customWidth="1"/>
+    <col min="5" max="5" width="16.21875" customWidth="1"/>
+    <col min="6" max="6" width="17.44140625" customWidth="1"/>
+    <col min="7" max="7" width="15.5546875" customWidth="1"/>
+    <col min="8" max="8" width="11.88671875" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="17.44140625" customWidth="1"/>
+    <col min="11" max="11" width="17.21875" customWidth="1"/>
+    <col min="12" max="12" width="17.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
@@ -542,29 +542,29 @@
       <c r="B2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="1">
+      <c r="C2" s="1">
         <v>0</v>
       </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
       <c r="E2" t="s">
         <v>12</v>
       </c>
       <c r="F2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" s="2">
+      <c r="G2" s="2">
         <v>0</v>
       </c>
-      <c r="J2" s="3">
+      <c r="H2" s="3">
         <v>0</v>
+      </c>
+      <c r="I2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" t="s">
+        <v>12</v>
       </c>
       <c r="K2" t="s">
         <v>12</v>

</xml_diff>